<commit_message>
Amplify E/I sociability baselines, matrix paths, and resting mood
Raise Extraversion (and mirror Introversion) so social expression reaches
spectrum edges more often at max intensity: stronger sociability baselines,
~2x signature mood→sociability matrix cells, and clearer belonging/arousal
resting mood. Sync JSON defaults, Excel generator/source, and loosen Phase-1
regression tolerances for the intentional drift.

Co-authored-by: astarrh <astarrh@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/personality_building_blocks.xlsx
+++ b/docs/personality_building_blocks.xlsx
@@ -2674,19 +2674,19 @@
         <v>-0.1</v>
       </c>
       <c r="S5" t="n">
-        <v>0.09</v>
+        <v>0.14</v>
       </c>
       <c r="T5" t="n">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.13</v>
       </c>
       <c r="V5" t="n">
         <v>0.15</v>
       </c>
       <c r="W5" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="X5" t="n">
         <v>0.06</v>
@@ -2725,7 +2725,7 @@
         <v>-0.25</v>
       </c>
       <c r="AJ5" t="n">
-        <v>-0.22</v>
+        <v>-0.39</v>
       </c>
       <c r="AK5" t="n">
         <v>0.11</v>
@@ -2740,13 +2740,13 @@
         <v>0.2</v>
       </c>
       <c r="AO5" t="n">
-        <v>-0.08</v>
+        <v>-0.13</v>
       </c>
       <c r="AP5" t="n">
         <v>0.09</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="6">
@@ -2809,19 +2809,19 @@
         <v>-0.13</v>
       </c>
       <c r="S6" t="n">
-        <v>0.02</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="T6" t="n">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.14</v>
+        <v>0.06</v>
       </c>
       <c r="V6" t="n">
         <v>0.12</v>
       </c>
       <c r="W6" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="X6" t="n">
         <v>0.02</v>
@@ -2860,7 +2860,7 @@
         <v>-0.1</v>
       </c>
       <c r="AJ6" t="n">
-        <v>-0.12</v>
+        <v>-0.29</v>
       </c>
       <c r="AK6" t="n">
         <v>-0.05</v>
@@ -2875,13 +2875,13 @@
         <v>0.1</v>
       </c>
       <c r="AO6" t="n">
-        <v>-0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="AP6" t="n">
         <v>0.02</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="7">
@@ -2944,19 +2944,19 @@
         <v>-0.1</v>
       </c>
       <c r="S7" t="n">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="T7" t="n">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.11</v>
+        <v>0.09</v>
       </c>
       <c r="V7" t="n">
         <v>0.11</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="X7" t="n">
         <v>0.02</v>
@@ -2995,7 +2995,7 @@
         <v>-0.2</v>
       </c>
       <c r="AJ7" t="n">
-        <v>-0.08</v>
+        <v>-0.25</v>
       </c>
       <c r="AK7" t="n">
         <v>-0.01</v>
@@ -3010,13 +3010,13 @@
         <v>0.08</v>
       </c>
       <c r="AO7" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.12</v>
       </c>
       <c r="AP7" t="n">
         <v>0.01</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="8">
@@ -3079,19 +3079,19 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="T8" t="n">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.04</v>
+        <v>0.16</v>
       </c>
       <c r="V8" t="n">
         <v>0.14</v>
       </c>
       <c r="W8" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="X8" t="n">
         <v>0.06</v>
@@ -3130,7 +3130,7 @@
         <v>-0.35</v>
       </c>
       <c r="AJ8" t="n">
-        <v>-0.18</v>
+        <v>-0.35</v>
       </c>
       <c r="AK8" t="n">
         <v>0.15</v>
@@ -3145,13 +3145,13 @@
         <v>0.18</v>
       </c>
       <c r="AO8" t="n">
-        <v>-0.12</v>
+        <v>-0.17</v>
       </c>
       <c r="AP8" t="n">
         <v>0.08</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="9">
@@ -3214,19 +3214,19 @@
         <v>-0.16</v>
       </c>
       <c r="S9" t="n">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="T9" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.12</v>
+        <v>0.08</v>
       </c>
       <c r="V9" t="n">
         <v>0.12</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.03</v>
+        <v>-0.01</v>
       </c>
       <c r="X9" t="n">
         <v>0.06</v>
@@ -3265,7 +3265,7 @@
         <v>0.05</v>
       </c>
       <c r="AJ9" t="n">
-        <v>-0.2</v>
+        <v>-0.37</v>
       </c>
       <c r="AK9" t="n">
         <v>0.06</v>
@@ -3280,13 +3280,13 @@
         <v>0.13</v>
       </c>
       <c r="AO9" t="n">
-        <v>-0.06</v>
+        <v>-0.11</v>
       </c>
       <c r="AP9" t="n">
         <v>0.04</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="10">
@@ -3349,19 +3349,19 @@
         <v>-0.19</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.03</v>
+        <v>0.02</v>
       </c>
       <c r="T10" t="n">
-        <v>-0.01</v>
+        <v>0.04</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.19</v>
+        <v>0.01</v>
       </c>
       <c r="V10" t="n">
         <v>0.09</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.05</v>
       </c>
       <c r="X10" t="n">
         <v>0.02</v>
@@ -3400,7 +3400,7 @@
         <v>0.2</v>
       </c>
       <c r="AJ10" t="n">
-        <v>-0.1</v>
+        <v>-0.27</v>
       </c>
       <c r="AK10" t="n">
         <v>-0.1</v>
@@ -3415,13 +3415,13 @@
         <v>0.03</v>
       </c>
       <c r="AO10" t="n">
-        <v>-0.01</v>
+        <v>-0.06</v>
       </c>
       <c r="AP10" t="n">
         <v>-0.03</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.31</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="11">
@@ -3484,19 +3484,19 @@
         <v>-0.16</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.01</v>
+        <v>0.04</v>
       </c>
       <c r="T11" t="n">
-        <v>-0.01</v>
+        <v>0.04</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.16</v>
+        <v>0.04</v>
       </c>
       <c r="V11" t="n">
         <v>0.08</v>
       </c>
       <c r="W11" t="n">
-        <v>-0.06</v>
+        <v>-0.04</v>
       </c>
       <c r="X11" t="n">
         <v>0.02</v>
@@ -3535,7 +3535,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ11" t="n">
-        <v>-0.06</v>
+        <v>-0.23</v>
       </c>
       <c r="AK11" t="n">
         <v>-0.06</v>
@@ -3550,13 +3550,13 @@
         <v>0.01</v>
       </c>
       <c r="AO11" t="n">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="AP11" t="n">
         <v>-0.04</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="12">
@@ -3619,19 +3619,19 @@
         <v>-0.13</v>
       </c>
       <c r="S12" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="T12" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.09</v>
+        <v>0.11</v>
       </c>
       <c r="V12" t="n">
         <v>0.11</v>
       </c>
       <c r="W12" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="X12" t="n">
         <v>0.06</v>
@@ -3670,7 +3670,7 @@
         <v>-0.05</v>
       </c>
       <c r="AJ12" t="n">
-        <v>-0.16</v>
+        <v>-0.33</v>
       </c>
       <c r="AK12" t="n">
         <v>0.1</v>
@@ -3685,13 +3685,13 @@
         <v>0.11</v>
       </c>
       <c r="AO12" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="AP12" t="n">
         <v>0.03</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="13">
@@ -3754,19 +3754,19 @@
         <v>-0.18</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.06</v>
+        <v>-0.11</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.02</v>
+        <v>-0.05</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.22</v>
+        <v>-0.32</v>
       </c>
       <c r="V13" t="n">
         <v>0.09</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="X13" t="n">
         <v>0.04</v>
@@ -3805,7 +3805,7 @@
         <v>0.15</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.1</v>
+        <v>0.27</v>
       </c>
       <c r="AK13" t="n">
         <v>0.03</v>
@@ -3820,13 +3820,13 @@
         <v>0.19</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="AP13" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="14">
@@ -3889,19 +3889,19 @@
         <v>-0.21</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.13</v>
+        <v>-0.18</v>
       </c>
       <c r="T14" t="n">
-        <v>-0.09</v>
+        <v>-0.12</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.29</v>
+        <v>-0.39</v>
       </c>
       <c r="V14" t="n">
         <v>0.06</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.14</v>
+        <v>-0.19</v>
       </c>
       <c r="X14" t="n">
         <v>0</v>
@@ -3940,7 +3940,7 @@
         <v>0.3</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.2</v>
+        <v>0.37</v>
       </c>
       <c r="AK14" t="n">
         <v>-0.13</v>
@@ -3955,13 +3955,13 @@
         <v>0.09</v>
       </c>
       <c r="AO14" t="n">
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="AP14" t="n">
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0.39</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="15">
@@ -4024,19 +4024,19 @@
         <v>-0.18</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.11</v>
+        <v>-0.16</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.09</v>
+        <v>-0.12</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.26</v>
+        <v>-0.36</v>
       </c>
       <c r="V15" t="n">
         <v>0.05</v>
       </c>
       <c r="W15" t="n">
-        <v>-0.13</v>
+        <v>-0.18</v>
       </c>
       <c r="X15" t="n">
         <v>0</v>
@@ -4075,7 +4075,7 @@
         <v>0.2</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.24</v>
+        <v>0.41</v>
       </c>
       <c r="AK15" t="n">
         <v>-0.09</v>
@@ -4090,13 +4090,13 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="AO15" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="AP15" t="n">
         <v>-0.01</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="16">
@@ -4159,19 +4159,19 @@
         <v>-0.15</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.04</v>
+        <v>-0.09</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.02</v>
+        <v>-0.05</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.19</v>
+        <v>-0.29</v>
       </c>
       <c r="V16" t="n">
         <v>0.08</v>
       </c>
       <c r="W16" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="X16" t="n">
         <v>0.04</v>
@@ -4210,7 +4210,7 @@
         <v>0.05</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0.14</v>
+        <v>0.31</v>
       </c>
       <c r="AK16" t="n">
         <v>0.07000000000000001</v>
@@ -4225,13 +4225,13 @@
         <v>0.17</v>
       </c>
       <c r="AO16" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="AP16" t="n">
         <v>0.06</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="17">
@@ -4294,19 +4294,19 @@
         <v>-0.12</v>
       </c>
       <c r="S17" t="n">
-        <v>-0.01</v>
+        <v>-0.06</v>
       </c>
       <c r="T17" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.17</v>
+        <v>-0.27</v>
       </c>
       <c r="V17" t="n">
         <v>0.12</v>
       </c>
       <c r="W17" t="n">
-        <v>-0.04</v>
+        <v>-0.09</v>
       </c>
       <c r="X17" t="n">
         <v>0.04</v>
@@ -4345,7 +4345,7 @@
         <v>-0.15</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="AK17" t="n">
         <v>0.08</v>
@@ -4360,13 +4360,13 @@
         <v>0.26</v>
       </c>
       <c r="AO17" t="n">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
       <c r="AP17" t="n">
         <v>0.12</v>
       </c>
       <c r="AQ17" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="18">
@@ -4429,19 +4429,19 @@
         <v>-0.15</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.08</v>
+        <v>-0.13</v>
       </c>
       <c r="T18" t="n">
-        <v>-0.04</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.24</v>
+        <v>-0.34</v>
       </c>
       <c r="V18" t="n">
         <v>0.09</v>
       </c>
       <c r="W18" t="n">
-        <v>-0.08</v>
+        <v>-0.13</v>
       </c>
       <c r="X18" t="n">
         <v>0</v>
@@ -4480,7 +4480,7 @@
         <v>0</v>
       </c>
       <c r="AJ18" t="n">
-        <v>0.18</v>
+        <v>0.35</v>
       </c>
       <c r="AK18" t="n">
         <v>-0.08</v>
@@ -4495,13 +4495,13 @@
         <v>0.16</v>
       </c>
       <c r="AO18" t="n">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="AP18" t="n">
         <v>0.05</v>
       </c>
       <c r="AQ18" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="19">
@@ -4564,19 +4564,19 @@
         <v>-0.12</v>
       </c>
       <c r="S19" t="n">
-        <v>-0.06</v>
+        <v>-0.11</v>
       </c>
       <c r="T19" t="n">
-        <v>-0.04</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.21</v>
+        <v>-0.31</v>
       </c>
       <c r="V19" t="n">
         <v>0.08</v>
       </c>
       <c r="W19" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.12</v>
       </c>
       <c r="X19" t="n">
         <v>0</v>
@@ -4615,7 +4615,7 @@
         <v>-0.1</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0.22</v>
+        <v>0.39</v>
       </c>
       <c r="AK19" t="n">
         <v>-0.04</v>
@@ -4630,13 +4630,13 @@
         <v>0.14</v>
       </c>
       <c r="AO19" t="n">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="AP19" t="n">
         <v>0.04</v>
       </c>
       <c r="AQ19" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="20">
@@ -4699,19 +4699,19 @@
         <v>-0.09</v>
       </c>
       <c r="S20" t="n">
-        <v>0.01</v>
+        <v>-0.04</v>
       </c>
       <c r="T20" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.14</v>
+        <v>-0.24</v>
       </c>
       <c r="V20" t="n">
         <v>0.11</v>
       </c>
       <c r="W20" t="n">
-        <v>-0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="X20" t="n">
         <v>0.04</v>
@@ -4750,7 +4750,7 @@
         <v>-0.25</v>
       </c>
       <c r="AJ20" t="n">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="AK20" t="n">
         <v>0.12</v>
@@ -4765,13 +4765,13 @@
         <v>0.24</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
       <c r="AP20" t="n">
         <v>0.11</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.28</v>
+        <v>0.33</v>
       </c>
     </row>
   </sheetData>
@@ -7128,19 +7128,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.03</v>
+        <v>-0.06</v>
       </c>
       <c r="D8" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F8" t="n">
         <v>-0.1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-0.05</v>
       </c>
     </row>
     <row r="9">
@@ -7277,19 +7277,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="C16" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E16" t="n">
         <v>0.05</v>
       </c>
       <c r="F16" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="17">
@@ -8303,7 +8303,7 @@
         <v>0.05</v>
       </c>
       <c r="D5" t="n">
-        <v>0.15</v>
+        <v>0.32</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -8325,7 +8325,7 @@
         <v>-0.05</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.15</v>
+        <v>-0.32</v>
       </c>
       <c r="E6" t="n">
         <v>0.03</v>
@@ -8518,13 +8518,13 @@
         <v>0.08</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="E16" t="n">
         <v>0.02</v>
       </c>
       <c r="F16" t="n">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="17">
@@ -8540,13 +8540,13 @@
         <v>0.02</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="E17" t="n">
         <v>-0.01</v>
       </c>
       <c r="F17" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Keep E/I retune in JSON only; deprecate Excel authoring
Revert spreadsheet/generator churn from the sociability amplification.
JSON remains the canonical default. Document Excel as deprecated and skip
JSON↔Excel parity tests.

Co-authored-by: astarrh <astarrh@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/personality_building_blocks.xlsx
+++ b/docs/personality_building_blocks.xlsx
@@ -2674,19 +2674,19 @@
         <v>-0.1</v>
       </c>
       <c r="S5" t="n">
-        <v>0.14</v>
+        <v>0.09</v>
       </c>
       <c r="T5" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="U5" t="n">
-        <v>0.13</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="V5" t="n">
         <v>0.15</v>
       </c>
       <c r="W5" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="X5" t="n">
         <v>0.06</v>
@@ -2725,7 +2725,7 @@
         <v>-0.25</v>
       </c>
       <c r="AJ5" t="n">
-        <v>-0.39</v>
+        <v>-0.22</v>
       </c>
       <c r="AK5" t="n">
         <v>0.11</v>
@@ -2740,13 +2740,13 @@
         <v>0.2</v>
       </c>
       <c r="AO5" t="n">
-        <v>-0.13</v>
+        <v>-0.08</v>
       </c>
       <c r="AP5" t="n">
         <v>0.09</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="6">
@@ -2809,19 +2809,19 @@
         <v>-0.13</v>
       </c>
       <c r="S6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="T6" t="n">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
       <c r="U6" t="n">
-        <v>0.06</v>
+        <v>-0.14</v>
       </c>
       <c r="V6" t="n">
         <v>0.12</v>
       </c>
       <c r="W6" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="X6" t="n">
         <v>0.02</v>
@@ -2860,7 +2860,7 @@
         <v>-0.1</v>
       </c>
       <c r="AJ6" t="n">
-        <v>-0.29</v>
+        <v>-0.12</v>
       </c>
       <c r="AK6" t="n">
         <v>-0.05</v>
@@ -2875,13 +2875,13 @@
         <v>0.1</v>
       </c>
       <c r="AO6" t="n">
-        <v>-0.08</v>
+        <v>-0.03</v>
       </c>
       <c r="AP6" t="n">
         <v>0.02</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="7">
@@ -2944,19 +2944,19 @@
         <v>-0.1</v>
       </c>
       <c r="S7" t="n">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
       <c r="T7" t="n">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
       <c r="U7" t="n">
-        <v>0.09</v>
+        <v>-0.11</v>
       </c>
       <c r="V7" t="n">
         <v>0.11</v>
       </c>
       <c r="W7" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
         <v>0.02</v>
@@ -2995,7 +2995,7 @@
         <v>-0.2</v>
       </c>
       <c r="AJ7" t="n">
-        <v>-0.25</v>
+        <v>-0.08</v>
       </c>
       <c r="AK7" t="n">
         <v>-0.01</v>
@@ -3010,13 +3010,13 @@
         <v>0.08</v>
       </c>
       <c r="AO7" t="n">
-        <v>-0.12</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="AP7" t="n">
         <v>0.01</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="8">
@@ -3079,19 +3079,19 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="T8" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="U8" t="n">
-        <v>0.16</v>
+        <v>-0.04</v>
       </c>
       <c r="V8" t="n">
         <v>0.14</v>
       </c>
       <c r="W8" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="X8" t="n">
         <v>0.06</v>
@@ -3130,7 +3130,7 @@
         <v>-0.35</v>
       </c>
       <c r="AJ8" t="n">
-        <v>-0.35</v>
+        <v>-0.18</v>
       </c>
       <c r="AK8" t="n">
         <v>0.15</v>
@@ -3145,13 +3145,13 @@
         <v>0.18</v>
       </c>
       <c r="AO8" t="n">
-        <v>-0.17</v>
+        <v>-0.12</v>
       </c>
       <c r="AP8" t="n">
         <v>0.08</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9">
@@ -3214,19 +3214,19 @@
         <v>-0.16</v>
       </c>
       <c r="S9" t="n">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
       <c r="T9" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="U9" t="n">
-        <v>0.08</v>
+        <v>-0.12</v>
       </c>
       <c r="V9" t="n">
         <v>0.12</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="X9" t="n">
         <v>0.06</v>
@@ -3265,7 +3265,7 @@
         <v>0.05</v>
       </c>
       <c r="AJ9" t="n">
-        <v>-0.37</v>
+        <v>-0.2</v>
       </c>
       <c r="AK9" t="n">
         <v>0.06</v>
@@ -3280,13 +3280,13 @@
         <v>0.13</v>
       </c>
       <c r="AO9" t="n">
-        <v>-0.11</v>
+        <v>-0.06</v>
       </c>
       <c r="AP9" t="n">
         <v>0.04</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="10">
@@ -3349,19 +3349,19 @@
         <v>-0.19</v>
       </c>
       <c r="S10" t="n">
-        <v>0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="T10" t="n">
-        <v>0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="U10" t="n">
-        <v>0.01</v>
+        <v>-0.19</v>
       </c>
       <c r="V10" t="n">
         <v>0.09</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.05</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="X10" t="n">
         <v>0.02</v>
@@ -3400,7 +3400,7 @@
         <v>0.2</v>
       </c>
       <c r="AJ10" t="n">
-        <v>-0.27</v>
+        <v>-0.1</v>
       </c>
       <c r="AK10" t="n">
         <v>-0.1</v>
@@ -3415,13 +3415,13 @@
         <v>0.03</v>
       </c>
       <c r="AO10" t="n">
-        <v>-0.06</v>
+        <v>-0.01</v>
       </c>
       <c r="AP10" t="n">
         <v>-0.03</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.29</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="11">
@@ -3484,19 +3484,19 @@
         <v>-0.16</v>
       </c>
       <c r="S11" t="n">
-        <v>0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="T11" t="n">
-        <v>0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="U11" t="n">
-        <v>0.04</v>
+        <v>-0.16</v>
       </c>
       <c r="V11" t="n">
         <v>0.08</v>
       </c>
       <c r="W11" t="n">
-        <v>-0.04</v>
+        <v>-0.06</v>
       </c>
       <c r="X11" t="n">
         <v>0.02</v>
@@ -3535,7 +3535,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ11" t="n">
-        <v>-0.23</v>
+        <v>-0.06</v>
       </c>
       <c r="AK11" t="n">
         <v>-0.06</v>
@@ -3550,13 +3550,13 @@
         <v>0.01</v>
       </c>
       <c r="AO11" t="n">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="AP11" t="n">
         <v>-0.04</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="12">
@@ -3619,19 +3619,19 @@
         <v>-0.13</v>
       </c>
       <c r="S12" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="T12" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="U12" t="n">
-        <v>0.11</v>
+        <v>-0.09</v>
       </c>
       <c r="V12" t="n">
         <v>0.11</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="X12" t="n">
         <v>0.06</v>
@@ -3670,7 +3670,7 @@
         <v>-0.05</v>
       </c>
       <c r="AJ12" t="n">
-        <v>-0.33</v>
+        <v>-0.16</v>
       </c>
       <c r="AK12" t="n">
         <v>0.1</v>
@@ -3685,13 +3685,13 @@
         <v>0.11</v>
       </c>
       <c r="AO12" t="n">
-        <v>-0.15</v>
+        <v>-0.1</v>
       </c>
       <c r="AP12" t="n">
         <v>0.03</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="13">
@@ -3754,19 +3754,19 @@
         <v>-0.18</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.11</v>
+        <v>-0.06</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.05</v>
+        <v>-0.02</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.32</v>
+        <v>-0.22</v>
       </c>
       <c r="V13" t="n">
         <v>0.09</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.15</v>
+        <v>-0.1</v>
       </c>
       <c r="X13" t="n">
         <v>0.04</v>
@@ -3805,7 +3805,7 @@
         <v>0.15</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.27</v>
+        <v>0.1</v>
       </c>
       <c r="AK13" t="n">
         <v>0.03</v>
@@ -3820,13 +3820,13 @@
         <v>0.19</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.19</v>
+        <v>0.14</v>
       </c>
       <c r="AP13" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="14">
@@ -3889,19 +3889,19 @@
         <v>-0.21</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.18</v>
+        <v>-0.13</v>
       </c>
       <c r="T14" t="n">
-        <v>-0.12</v>
+        <v>-0.09</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.39</v>
+        <v>-0.29</v>
       </c>
       <c r="V14" t="n">
         <v>0.06</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.19</v>
+        <v>-0.14</v>
       </c>
       <c r="X14" t="n">
         <v>0</v>
@@ -3940,7 +3940,7 @@
         <v>0.3</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.37</v>
+        <v>0.2</v>
       </c>
       <c r="AK14" t="n">
         <v>-0.13</v>
@@ -3955,13 +3955,13 @@
         <v>0.09</v>
       </c>
       <c r="AO14" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="AP14" t="n">
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0.44</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="15">
@@ -4024,19 +4024,19 @@
         <v>-0.18</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.16</v>
+        <v>-0.11</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.12</v>
+        <v>-0.09</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.36</v>
+        <v>-0.26</v>
       </c>
       <c r="V15" t="n">
         <v>0.05</v>
       </c>
       <c r="W15" t="n">
-        <v>-0.18</v>
+        <v>-0.13</v>
       </c>
       <c r="X15" t="n">
         <v>0</v>
@@ -4075,7 +4075,7 @@
         <v>0.2</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.41</v>
+        <v>0.24</v>
       </c>
       <c r="AK15" t="n">
         <v>-0.09</v>
@@ -4090,13 +4090,13 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="AO15" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="AP15" t="n">
         <v>-0.01</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="16">
@@ -4159,19 +4159,19 @@
         <v>-0.15</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.09</v>
+        <v>-0.04</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.05</v>
+        <v>-0.02</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.29</v>
+        <v>-0.19</v>
       </c>
       <c r="V16" t="n">
         <v>0.08</v>
       </c>
       <c r="W16" t="n">
-        <v>-0.14</v>
+        <v>-0.09</v>
       </c>
       <c r="X16" t="n">
         <v>0.04</v>
@@ -4210,7 +4210,7 @@
         <v>0.05</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0.31</v>
+        <v>0.14</v>
       </c>
       <c r="AK16" t="n">
         <v>0.07000000000000001</v>
@@ -4225,13 +4225,13 @@
         <v>0.17</v>
       </c>
       <c r="AO16" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="AP16" t="n">
         <v>0.06</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0.38</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="17">
@@ -4294,19 +4294,19 @@
         <v>-0.12</v>
       </c>
       <c r="S17" t="n">
-        <v>-0.06</v>
+        <v>-0.01</v>
       </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.27</v>
+        <v>-0.17</v>
       </c>
       <c r="V17" t="n">
         <v>0.12</v>
       </c>
       <c r="W17" t="n">
-        <v>-0.09</v>
+        <v>-0.04</v>
       </c>
       <c r="X17" t="n">
         <v>0.04</v>
@@ -4345,7 +4345,7 @@
         <v>-0.15</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="AK17" t="n">
         <v>0.08</v>
@@ -4360,13 +4360,13 @@
         <v>0.26</v>
       </c>
       <c r="AO17" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="AP17" t="n">
         <v>0.12</v>
       </c>
       <c r="AQ17" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="18">
@@ -4429,19 +4429,19 @@
         <v>-0.15</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.13</v>
+        <v>-0.08</v>
       </c>
       <c r="T18" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.34</v>
+        <v>-0.24</v>
       </c>
       <c r="V18" t="n">
         <v>0.09</v>
       </c>
       <c r="W18" t="n">
-        <v>-0.13</v>
+        <v>-0.08</v>
       </c>
       <c r="X18" t="n">
         <v>0</v>
@@ -4480,7 +4480,7 @@
         <v>0</v>
       </c>
       <c r="AJ18" t="n">
-        <v>0.35</v>
+        <v>0.18</v>
       </c>
       <c r="AK18" t="n">
         <v>-0.08</v>
@@ -4495,13 +4495,13 @@
         <v>0.16</v>
       </c>
       <c r="AO18" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="AP18" t="n">
         <v>0.05</v>
       </c>
       <c r="AQ18" t="n">
-        <v>0.39</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="19">
@@ -4564,19 +4564,19 @@
         <v>-0.12</v>
       </c>
       <c r="S19" t="n">
-        <v>-0.11</v>
+        <v>-0.06</v>
       </c>
       <c r="T19" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.31</v>
+        <v>-0.21</v>
       </c>
       <c r="V19" t="n">
         <v>0.08</v>
       </c>
       <c r="W19" t="n">
-        <v>-0.12</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="X19" t="n">
         <v>0</v>
@@ -4615,7 +4615,7 @@
         <v>-0.1</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0.39</v>
+        <v>0.22</v>
       </c>
       <c r="AK19" t="n">
         <v>-0.04</v>
@@ -4630,13 +4630,13 @@
         <v>0.14</v>
       </c>
       <c r="AO19" t="n">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
       <c r="AP19" t="n">
         <v>0.04</v>
       </c>
       <c r="AQ19" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="20">
@@ -4699,19 +4699,19 @@
         <v>-0.09</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.04</v>
+        <v>0.01</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.24</v>
+        <v>-0.14</v>
       </c>
       <c r="V20" t="n">
         <v>0.11</v>
       </c>
       <c r="W20" t="n">
-        <v>-0.08</v>
+        <v>-0.03</v>
       </c>
       <c r="X20" t="n">
         <v>0.04</v>
@@ -4750,7 +4750,7 @@
         <v>-0.25</v>
       </c>
       <c r="AJ20" t="n">
-        <v>0.29</v>
+        <v>0.12</v>
       </c>
       <c r="AK20" t="n">
         <v>0.12</v>
@@ -4765,13 +4765,13 @@
         <v>0.24</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.13</v>
+        <v>0.08</v>
       </c>
       <c r="AP20" t="n">
         <v>0.11</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.33</v>
+        <v>0.28</v>
       </c>
     </row>
   </sheetData>
@@ -7128,19 +7128,19 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="D8" t="n">
         <v>-0.1</v>
       </c>
-      <c r="C8" t="n">
-        <v>-0.06</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-0.2</v>
-      </c>
       <c r="E8" t="n">
         <v>0.02</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="9">
@@ -7277,19 +7277,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="C16" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>0.05</v>
       </c>
       <c r="F16" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="17">
@@ -8303,7 +8303,7 @@
         <v>0.05</v>
       </c>
       <c r="D5" t="n">
-        <v>0.32</v>
+        <v>0.15</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -8325,7 +8325,7 @@
         <v>-0.05</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.32</v>
+        <v>-0.15</v>
       </c>
       <c r="E6" t="n">
         <v>0.03</v>
@@ -8518,13 +8518,13 @@
         <v>0.08</v>
       </c>
       <c r="D16" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="E16" t="n">
         <v>0.02</v>
       </c>
       <c r="F16" t="n">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="17">
@@ -8540,13 +8540,13 @@
         <v>0.02</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.15</v>
+        <v>-0.1</v>
       </c>
       <c r="E17" t="n">
         <v>-0.01</v>
       </c>
       <c r="F17" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="18">

</xml_diff>